<commit_message>
added bison hunting dates
</commit_message>
<xml_diff>
--- a/data/raw/hunting_seasons.xlsx
+++ b/data/raw/hunting_seasons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\billy.DESKTOP-6FIO124\Documents\Master Thesis\raven_movement\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{402FFD4F-40A1-46E7-86FC-97C968E28C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{604C78C6-86D4-4350-B66F-5C0A25A5A423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25110" yWindow="3690" windowWidth="21600" windowHeight="11715" xr2:uid="{F8409187-CC4D-4331-8FBB-89995D232744}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{F8409187-CC4D-4331-8FBB-89995D232744}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>year</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>md_end</t>
+  </si>
+  <si>
+    <t>bison</t>
   </si>
 </sst>
 </file>
@@ -423,13 +426,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78DD8620-79C6-42CB-9ED7-BB7F6B1215B3}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="4" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -442,8 +445,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2019</v>
       </c>
@@ -456,8 +462,11 @@
       <c r="D2" s="1">
         <v>43786</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2" s="1">
+        <v>43884</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2020</v>
       </c>
@@ -470,8 +479,11 @@
       <c r="D3" s="1">
         <v>44150</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E3" s="1">
+        <v>44221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -484,8 +496,11 @@
       <c r="D4" s="1">
         <v>44514</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E4" s="1">
+        <v>44642</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2022</v>
       </c>
@@ -498,8 +513,11 @@
       <c r="D5" s="1">
         <v>44878</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E5" s="1">
+        <v>44903</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2023</v>
       </c>
@@ -512,8 +530,11 @@
       <c r="D6" s="1">
         <v>45242</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6" s="1">
+        <v>45375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -526,8 +547,11 @@
       <c r="D7" s="1">
         <v>45613</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7" s="1">
+        <v>45727</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2025</v>
       </c>

</xml_diff>